<commit_message>
feat(F-NAR-018): avis2 — étalon structurel, AUT-001, COL-001, deux ATOM
Ingest avis2.txt. TREE-AUT-001 : oral plus lié, morale vécue.
TREE-COL-001 : pomme qui s'échappe, T3 ramasse/attendre/invente.
ATOM dessin du soleil et boîte trop haute : plus de récap Bravo.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.001-05.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.001-05.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon, fin d’après-midi</t>
+          <t>salon, fin d'après-midi</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah finit un dessin. Un soleil. Une maison. Elle dit sa joie. Elle le montre à papa, puis à maman.</t>
+          <t>Sarah dessine la maison pour maman, qui n'est pas rentrée. Le crayon jaune casse. Elle attend, puis montre.</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Dans le salon, un rayon traverse la poussière. Les crayons dorment dans leur boîte en fer. La boîte est froide et un peu cabossée. Le tapis sent la laine. Un coussin a glissé sous la table. La pendule fait tic, tout bas. Papa coud un bouton, près de la fenêtre. Maman n'est pas encore rentrée. Dehors, on entend un vélo, très loin. Sarah, tu as choisi une feuille ? Oui. La grande, blanche. Tu as de la place pour un soleil. En ce moment, Sarah est assise au bas du canapé. Elle pose la feuille sur le tapis. Le crayon jaune fait un bruit sec sur le papier. Un soleil rond. Des rayons. Une petite maison. Une porte. Deux fenêtres. Papa, j'ai fini. Montre-moi, tout doucement. Sarah tend le dessin. Parce qu'elle a fini, ses joues deviennent chaudes. Son ventre est léger. Un sourire arrive. Je suis contente. C'est de la joie. Tu as nommé ta joie. Bravo, Sarah. On peut partager le dessin ? Oui. On le regarde ensemble. Papa le tient par les bords. Il ne plie pas la feuille. Le soleil est très jaune. C'est notre maison. La porte d'entrée clique. Maman pose son sac. Je rentre. Ça sent les crayons. Maman, viens voir. Tu me montres ? Sarah attend que maman s'assoie. Puis elle tend le dessin, sans bousculer. Merci, Sarah. Tu partages ta joie. C'est gentil. Je suis contente. C'est de la joie, dans le salon. Tu as encore envie de raconter ton dessin ? Oui. Le soleil, et la maison.</t>
+          <t>Un rayon traverse la poussière du salon. Les crayons dorment dans leur boîte en fer. La boîte est froide, un peu cabossée. Le tapis sent la laine. Un coussin a glissé sous la table. La pendule fait tic, tout bas. Papa coud un bouton près de la fenêtre. Maman n'est pas encore rentrée. Dehors, un vélo passe, très loin. Sarah, tu as choisi une feuille ? La grande, blanche. C'est pour maman. Elle va rentrer bientôt. En ce moment, Sarah s'assoit au bas du canapé. Elle pose la feuille sur le tapis. Le crayon jaune fait un bruit sec. Un soleil rond, puis des rayons. Une petite maison, une porte, deux fenêtres. Le crayon jaune casse, net. Oh. Il en reste un bout. Sarah souffle la mine tombée sur le tapis. Elle finit le toit avec le bout. Un rayon manque encore, tout petit. Maman va voir le trou ? Elle verra la maison, d'abord. Sarah pose le bout de crayon. La porte d'entrée clique. Maman pose son sac. Je rentre. Ça sent les crayons. Attends. Sarah attend que maman s'assoie. Ses joues sont chaudes. Elle tend la feuille, sans bousculer. C'est notre maison. Je suis contente. Merci, Sarah. Le soleil est très jaune. On le met où ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Dans le salon, un rayon traverse la poussière. Les crayons dorment dans leur boîte en fer. La boîte est froide et un peu cabossée. Le tapis sent la laine. Un coussin a glissé sous la table. La pendule fait tic, tout bas. Papa coud un bouton, près de la fenêtre. Maman n'est pas encore rentrée. Dehors, on entend un vélo, très loin. Sarah, tu as choisi une feuille ? Oui. La grande, blanche. Tu as de la place pour un soleil. En ce moment, Sarah est assise au bas du canapé. Elle pose la feuille sur le tapis. Le crayon jaune fait un bruit sec sur le papier. Un soleil rond. Des rayons. Une petite maison. Une porte. Deux fenêtres. Papa, j'ai fini. Montre-moi, tout doucement. Sarah tend le dessin. Parce qu'elle a fini, ses joues deviennent chaudes. Son ventre est léger. Un sourire arrive. Je suis contente. C'est de la joie. Tu as nommé ta joie. Bravo, Sarah. On peut partager le dessin ? Oui. On le regarde ensemble. Papa le tient par les bords. Il ne plie pas la feuille. Le soleil est très jaune. C'est notre maison. La porte d'entrée clique. Maman pose son sac. Je rentre. Ça sent les crayons. Maman, viens voir. Tu me montres ? Sarah attend que maman s'assoie. Puis elle tend le dessin, sans bousculer. Merci, Sarah. Tu partages ta joie. C'est gentil. Je suis contente. C'est de la joie, dans le salon. Tu as encore envie de raconter ton dessin ? Oui. Le soleil, et la maison.</t>
+          <t>Un rayon traverse la poussière du salon. Les crayons dorment dans leur boîte en fer. La boîte est froide, un peu cabossée. Le tapis sent la laine. Un coussin a glissé sous la table. La pendule fait tic, tout bas. Papa coud un bouton près de la fenêtre. Maman n'est pas encore rentrée. Dehors, un vélo passe, très loin. Sarah, tu as choisi une feuille ? La grande, blanche. C'est pour maman. Elle va rentrer bientôt. En ce moment, Sarah s'assoit au bas du canapé. Elle pose la feuille sur le tapis. Le crayon jaune fait un bruit sec. Un soleil rond, puis des rayons. Une petite maison, une porte, deux fenêtres. Le crayon jaune casse, net. Oh. Il en reste un bout. Sarah souffle la mine tombée sur le tapis. Elle finit le toit avec le bout. Un rayon manque encore, tout petit. Maman va voir le trou ? Elle verra la maison, d'abord. Sarah pose le bout de crayon. La porte d'entrée clique. Maman pose son sac. Je rentre. Ça sent les crayons. Attends. Sarah attend que maman s'assoie. Ses joues sont chaudes. Elle tend la feuille, sans bousculer. C'est notre maison. Je suis contente. Merci, Sarah. Le soleil est très jaune. On le met où ?</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
         <v>0.96</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.12</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1324,52 +1324,46 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Dans le salon, un rayon traverse la poussière.
+          <t>narrateur|Un rayon traverse la poussière du salon.
 narrateur|Les crayons dorment dans leur boîte en fer.
-narrateur|La boîte est froide et un peu cabossée.
+narrateur|La boîte est froide, un peu cabossée.
 narrateur|Le tapis sent la laine.
 narrateur|Un coussin a glissé sous la table.
 narrateur|La pendule fait tic, tout bas.
-narrateur|Papa coud un bouton, près de la fenêtre.
+narrateur|Papa coud un bouton près de la fenêtre.
 narrateur|Maman n'est pas encore rentrée.
-narrateur|Dehors, on entend un vélo, très loin.
+narrateur|Dehors, un vélo passe, très loin.
 papa|Sarah, tu as choisi une feuille ?
-enfant-f|Oui. La grande, blanche.
-papa|Tu as de la place pour un soleil.
-narrateur|En ce moment, Sarah est assise au bas du canapé.
+enfant-f|La grande, blanche.
+enfant-f|C'est pour maman.
+papa|Elle va rentrer bientôt.
+narrateur|En ce moment, Sarah s'assoit au bas du canapé.
 narrateur|Elle pose la feuille sur le tapis.
-narrateur|Le crayon jaune fait un bruit sec sur le papier.
-narrateur|Un soleil rond. Des rayons. Une petite maison.
-narrateur|Une porte. Deux fenêtres.
-enfant-f|Papa, j'ai fini.
-papa|Montre-moi, tout doucement.
-narrateur|Sarah tend le dessin.
-narrateur|Parce qu'elle a fini, ses joues deviennent chaudes.
-narrateur|Son ventre est léger.
-narrateur|Un sourire arrive.
-enfant-f|Je suis contente.
-papa|C'est de la joie.
-papa|Tu as nommé ta joie.
-papa|Bravo, Sarah.
-enfant-f|On peut partager le dessin ?
-papa|Oui. On le regarde ensemble.
-narrateur|Papa le tient par les bords.
-narrateur|Il ne plie pas la feuille.
-papa|Le soleil est très jaune.
-enfant-f|C'est notre maison.
+narrateur|Le crayon jaune fait un bruit sec.
+narrateur|Un soleil rond, puis des rayons.
+narrateur|Une petite maison, une porte, deux fenêtres.
+narrateur|Le crayon jaune casse, net.
+enfant-f|Oh.
+papa|Il en reste un bout.
+narrateur|Sarah souffle la mine tombée sur le tapis.
+narrateur|Elle finit le toit avec le bout.
+narrateur|Un rayon manque encore, tout petit.
+enfant-f|Maman va voir le trou ?
+papa|Elle verra la maison, d'abord.
+narrateur|Sarah pose le bout de crayon.
 narrateur|La porte d'entrée clique.
 narrateur|Maman pose son sac.
-maman|Je rentre. Ça sent les crayons.
-enfant-f|Maman, viens voir.
-maman|Tu me montres ?
+maman|Je rentre.
+maman|Ça sent les crayons.
+enfant-f|Attends.
 narrateur|Sarah attend que maman s'assoie.
-narrateur|Puis elle tend le dessin, sans bousculer.
+narrateur|Ses joues sont chaudes.
+narrateur|Elle tend la feuille, sans bousculer.
+enfant-f|C'est notre maison.
+enfant-f|Je suis contente.
 maman|Merci, Sarah.
-maman|Tu partages ta joie. C'est gentil.
-enfant-f|Je suis contente.
-maman|C'est de la joie, dans le salon.
-papa|Tu as encore envie de raconter ton dessin ?
-enfant-f|Oui. Le soleil, et la maison.</t>
+papa|Le soleil est très jaune.
+maman|On le met où ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1401,42 +1395,42 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>Sarah sourit, la feuille encore chaude. Que dit-elle ?</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Sarah sourit, la feuille encore chaude. Que dit-elle ?</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Ninon sourit. Que dit-elle ?</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>contente</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>contente | je suis contente | joie</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Oui, c'est la bonne réponse.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Tu étais presque.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
           <t>Sarah sourit. Que dit-elle ?</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Sarah sourit. Que dit-elle ?</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Ninon sourit. Que dit-elle ?</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>contente</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>contente | je suis contente | joie | de la joie | partager</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Oui, c'est la bonne réponse.</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Tu étais presque.</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Ninon sent de la joie. Que dit-elle ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1478,14 +1472,14 @@
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
         <v>0.9</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.28</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1557,7 +1551,8 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Sarah sourit. Que dit-elle ?</t>
+          <t>narrateur|Sarah sourit, la feuille encore chaude.
+maman|Que dit-elle ?</t>
         </is>
       </c>
     </row>
@@ -1584,12 +1579,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah repose le dessin sur la table basse. C'est de la joie. Oui. Tu es contente. Tu as partagé avec papa et avec moi. Tu as fini de montrer ton dessin ? Oui. Les crayons rentrent dans la boîte, un par un. Le soleil de la feuille reste bien visible.</t>
+          <t>Maman tient la feuille par les bords. Elle ne plie pas le soleil. Le vrai soleil est à la fenêtre. On va le voir ensemble ? Ils se lèvent. Le sac de maman reste près de la porte. J'apporte la pince à linge ? Oui. Papa prend une pince sur le radiateur. La pince est un peu tiède. Comme le rayon.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah repose le dessin sur la table basse. C'est de la joie. Oui. Tu es contente. Tu as partagé avec papa et avec moi. Tu as fini de montrer ton dessin ? Oui. Les crayons rentrent dans la boîte, un par un. Le soleil de la feuille reste bien visible.</t>
+          <t>Maman tient la feuille par les bords. Elle ne plie pas le soleil. Le vrai soleil est à la fenêtre. On va le voir ensemble ? Ils se lèvent. Le sac de maman reste près de la porte. J'apporte la pince à linge ? Oui. Papa prend une pince sur le radiateur. La pince est un peu tiède. Comme le rayon.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1652,7 +1647,7 @@
         <v>0.96</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.22</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1728,14 +1723,17 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah repose le dessin sur la table basse.
-enfant-f|C'est de la joie.
-maman|Oui. Tu es contente.
-maman|Tu as partagé avec papa et avec moi.
-papa|Tu as fini de montrer ton dessin ?
+          <t>narrateur|Maman tient la feuille par les bords.
+narrateur|Elle ne plie pas le soleil.
+enfant-f|Le vrai soleil est à la fenêtre.
+maman|On va le voir ensemble ?
+narrateur|Ils se lèvent.
+narrateur|Le sac de maman reste près de la porte.
+papa|J'apporte la pince à linge ?
 enfant-f|Oui.
-narrateur|Les crayons rentrent dans la boîte, un par un.
-narrateur|Le soleil de la feuille reste bien visible.</t>
+narrateur|Papa prend une pince sur le radiateur.
+narrateur|La pince est un peu tiède.
+enfant-f|Comme le rayon.</t>
         </is>
       </c>
     </row>
@@ -1762,12 +1760,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sarah ferme la boîte en fer. Ça fait un petit clac. On le met près de la fenêtre ? Oui. Pour le voir. Tu as bien invité. Je suis contente. La joie est là, près du dessin. Le rayon a bougé un peu sur le tapis. Ils restent au salon, tout près.</t>
+          <t>Ils collent le dessin contre la vitre. La pince tient le coin. Dehors, le vrai soleil est plus pâle. Le mien est plus rond. Le tien attendait, sur le tapis. Le crayon cassé reste dans la boîte. Sarah range les autres crayons, un par un. Le jaune cassé rentre le dernier. La boîte fait un petit clac. On laisse le dessin pour la nuit ? Oui. Il garde la fenêtre.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sarah ferme la boîte en fer. Ça fait un petit clac. On le met près de la fenêtre ? Oui. Pour le voir. Tu as bien invité. Je suis contente. La joie est là, près du dessin. Le rayon a bougé un peu sur le tapis. Ils restent au salon, tout près.</t>
+          <t>Ils collent le dessin contre la vitre. La pince tient le coin. Dehors, le vrai soleil est plus pâle. Le mien est plus rond. Le tien attendait, sur le tapis. Le crayon cassé reste dans la boîte. Sarah range les autres crayons, un par un. Le jaune cassé rentre le dernier. La boîte fait un petit clac. On laisse le dessin pour la nuit ? Oui. Il garde la fenêtre.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1830,7 +1828,7 @@
         <v>0.96</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.22</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1902,15 +1900,23 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sarah ferme la boîte en fer.
-narrateur|Ça fait un petit clac.
-maman|On le met près de la fenêtre ?
-enfant-f|Oui. Pour le voir.
-papa|Tu as bien invité.
-enfant-f|Je suis contente.
-maman|La joie est là, près du dessin.
-narrateur|Le rayon a bougé un peu sur le tapis.
-narrateur|Ils restent au salon, tout près.</t>
+          <t>narrateur|Ils collent le dessin contre la vitre.
+narrateur|La pince tient le coin.
+narrateur|Dehors, le vrai soleil est plus pâle.
+enfant-f|Le mien est plus rond.
+maman|Le tien attendait, sur le tapis.
+papa|Le crayon cassé reste dans la boîte.
+narrateur|Sarah range les autres crayons, un par un.
+narrateur|Le jaune cassé rentre le dernier.
+narrateur|La boîte fait un petit clac.
+papa|On laisse le dessin pour la nuit ?
+enfant-f|Oui.
+enfant-f|Il garde la fenêtre.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>clic</t>
         </is>
       </c>
     </row>
@@ -1937,12 +1943,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis contente. On a partagé le dessin. Bravo, Sarah.</t>
+          <t>Le rayon a bougé sur le tapis. Sur la vitre, la maison reste. Maman l'a vue. Je la verrai encore demain. Le sac de maman sent encore le dehors. Ils restent au salon, tout près.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis contente. On a partagé le dessin. Bravo, Sarah.</t>
+          <t>Le rayon a bougé sur le tapis. Sur la vitre, la maison reste. Maman l'a vue. Je la verrai encore demain. Le sac de maman sent encore le dehors. Ils restent au salon, tout près.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2005,7 +2011,7 @@
         <v>0.92</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.22</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2077,9 +2083,12 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai dit : je suis contente.
-enfant-f|On a partagé le dessin.
-papa|Bravo, Sarah.</t>
+          <t>narrateur|Le rayon a bougé sur le tapis.
+narrateur|Sur la vitre, la maison reste.
+enfant-f|Maman l'a vue.
+maman|Je la verrai encore demain.
+narrateur|Le sac de maman sent encore le dehors.
+narrateur|Ils restent au salon, tout près.</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2164,6 +2173,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.001-05 Sarah et le dessin du soleil
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.001-05.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.001-05.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon, fin d'après-midi</t>
+          <t>salon, fin d'après-midi, tapis, poussière, crayons, feuille, vitre, pince, gomme, fenêtre, table basse</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah dessine la maison pour maman, qui n'est pas rentrée. Le crayon jaune casse. Elle attend, puis montre.</t>
+          <t>La laine du tapis sent le soleil. Près de la feuille, un éclat de gomme luit. Sarah veut montrer le soleil à maman, maintenant. Maman n'est pas rentrée. Le crayon jaune casse. Sourire parti. Papa s'accroupit. Elle attend, puis montre : je suis contente. Merci vécu. Deuxième ruse : la feuille se plie à la vitre. Elle refuse de foncer. Un éclat de gomme tient sur le papier.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un rayon traverse la poussière du salon. Les crayons dorment dans leur boîte en fer. La boîte est froide, un peu cabossée. Le tapis sent la laine. Un coussin a glissé sous la table. La pendule fait tic, tout bas. Papa coud un bouton près de la fenêtre. Maman n'est pas encore rentrée. Dehors, un vélo passe, très loin. Sarah, tu as choisi une feuille ? La grande, blanche. C'est pour maman. Elle va rentrer bientôt. En ce moment, Sarah s'assoit au bas du canapé. Elle pose la feuille sur le tapis. Le crayon jaune fait un bruit sec. Un soleil rond, puis des rayons. Une petite maison, une porte, deux fenêtres. Le crayon jaune casse, net. Oh. Il en reste un bout. Sarah souffle la mine tombée sur le tapis. Elle finit le toit avec le bout. Un rayon manque encore, tout petit. Maman va voir le trou ? Elle verra la maison, d'abord. Sarah pose le bout de crayon. La porte d'entrée clique. Maman pose son sac. Je rentre. Ça sent les crayons. Attends. Sarah attend que maman s'assoie. Ses joues sont chaudes. Elle tend la feuille, sans bousculer. C'est notre maison. Je suis contente. Merci, Sarah. Le soleil est très jaune. On le met où ?</t>
+          <t>La laine du tapis sent le soleil. Ça sent la laine, papa. Tu la sens, la laine chaude ? Oui, papa. Sarah connaît ce salon, ses recoins. Cette fin d'après-midi, un coin brille autrement. La poussière danse près de la table basse. Elle danse, papa. Tu la vois, près des crayons ? Oui. La boîte en fer est froide, un peu cabossée. Elle claque. Sarah ouvre la boîte près des genoux. Les crayons roulent, un petit bruit. Sarah, tu as choisi une feuille ? La grande, blanche. C'est pour maman. Maman n'est pas rentrée. Je lui fais un soleil. Près de la feuille, un éclat de gomme luit. Il brille, papa. Tu le vois, le petit point ? Oui, un grain blanc. Papa coud un bouton, près de la fenêtre. Dehors, un vélo passe, très loin. Maman revient ? Bientôt. En ce moment, Sarah s'assoit au bas du canapé. Elle pose la feuille sur le tapis. Le crayon jaune fait un bruit sec. Un soleil rond ! Des rayons partent, puis une petite maison. Une porte, deux fenêtres. C'est notre maison. Tu as de la place, Sarah ? Oui, papa. Sarah appuie trop fort, trop vite. Le crayon jaune casse, net. Oh. Il en reste un bout. La mine tombe sur le tapis. Maman va voir le trou ? Elle verra la maison. Sarah veut finir, tout de suite. Je montre, maintenant ! Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois le bout, Sarah ? Oui, papa. L'éclat de gomme tremble, puis tient. Sarah finit le toit avec le bout. Un rayon manque. La maison est là. La porte clique, dans le couloir. Maman pose son sac. Je rentre. Ça sent les crayons. Attends. Sarah attend que maman s'assoie. Ses joues sont chaudes. Elle tend la feuille, sans bousculer. C'est notre maison. Je suis contente. Le soleil est très jaune. On le met où ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un rayon traverse la poussière du salon. Les crayons dorment dans leur boîte en fer. La boîte est froide, un peu cabossée. Le tapis sent la laine. Un coussin a glissé sous la table. La pendule fait tic, tout bas. Papa coud un bouton près de la fenêtre. Maman n'est pas encore rentrée. Dehors, un vélo passe, très loin. Sarah, tu as choisi une feuille ? La grande, blanche. C'est pour maman. Elle va rentrer bientôt. En ce moment, Sarah s'assoit au bas du canapé. Elle pose la feuille sur le tapis. Le crayon jaune fait un bruit sec. Un soleil rond, puis des rayons. Une petite maison, une porte, deux fenêtres. Le crayon jaune casse, net. Oh. Il en reste un bout. Sarah souffle la mine tombée sur le tapis. Elle finit le toit avec le bout. Un rayon manque encore, tout petit. Maman va voir le trou ? Elle verra la maison, d'abord. Sarah pose le bout de crayon. La porte d'entrée clique. Maman pose son sac. Je rentre. Ça sent les crayons. Attends. Sarah attend que maman s'assoie. Ses joues sont chaudes. Elle tend la feuille, sans bousculer. C'est notre maison. Je suis contente. Merci, Sarah. Le soleil est très jaune. On le met où ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La laine du tapis sent le soleil. Ça sent la laine, papa. Tu la sens, la laine chaude ? Oui, papa. Sarah connaît ce salon, ses recoins. Cette fin d'après-midi, un coin brille autrement. La poussière danse près de la table basse. Elle danse, papa. Tu la vois, près des crayons ? Oui. La boîte en fer est froide, un peu cabossée. Elle claque. Sarah ouvre la boîte près des genoux. Les crayons roulent, un petit bruit. Sarah, tu as choisi une feuille ? La grande, blanche. C'est pour maman. Maman n'est pas rentrée. Je lui fais un soleil. Près de la feuille, un &lt;emphasis level="moderate"&gt;éclat de gomme&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un grain blanc. Papa coud un bouton, près de la fenêtre. Dehors, un vélo passe, très loin. Maman revient ? Bientôt. En ce moment, Sarah s'assoit au bas du canapé. Elle pose la feuille sur le tapis. Le crayon jaune fait un bruit sec. Un soleil rond ! Des rayons partent, puis une petite maison. Une porte, deux fenêtres. C'est notre maison. Tu as de la place, Sarah ? Oui, papa. Sarah appuie trop fort, trop vite. Le crayon jaune casse, net. Oh. Il en reste un bout. La mine tombe sur le tapis. Maman va voir le trou ? Elle verra la maison. Sarah veut finir, tout de suite. Je montre, maintenant ! Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois le bout, Sarah ? Oui, papa. L'éclat de gomme tremble, puis tient. Sarah finit le toit avec le bout. Un rayon manque. La maison est là. La porte clique, dans le couloir. Maman pose son sac. Je rentre. Ça sent les crayons. Attends. Sarah attend que maman s'assoie. Ses joues sont chaudes. Elle tend la feuille, sans bousculer. C'est notre maison. Je suis contente. Le soleil est très jaune. On le met où ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Ninon est dans le salon avec papa. Elle a fini un dessin. Un soleil jaune. Une petite maison. Ninon sent ses joues chaudes. Son ventre est léger. Un sourire arrive. Ninon dit : je suis &lt;emphasis&gt;content&lt;/emphasis&gt;e. Papa dit : c'est de la joie. Ninon tend le dessin. Elle dit : on peut partager. Papa le regarde. Il sourit. Plus tard, maman rentre. Ninon montre le dessin à maman aussi. Elle partage sa joie sans bousculer. Maman dit : merci Ninon. Ninon dit encore : je suis contente. La joie est là, dans le salon. Papa et maman sont près d'elle. [pause]</t>
+          <t>La laine du tapis sent le soleil. Ça sent la laine, papa. Tu la sens, la laine chaude ? Oui, papa. Sarah connaît ce salon, ses recoins. Cette fin d'après-midi, un coin brille autrement. La poussière danse près de la table basse. Elle danse, papa. Tu la vois, près des crayons ? Oui. La boîte en fer est froide, un peu cabossée. Elle claque. Sarah ouvre la boîte près des genoux. Les crayons roulent, un petit bruit. Sarah, tu as choisi une feuille ? La grande, blanche. C'est pour maman. Maman n'est pas rentrée. Je lui fais un soleil. Près de la feuille, un &lt;emphasis&gt;éclat de gomme&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un grain blanc. Papa coud un bouton, près de la fenêtre. Dehors, un vélo passe, très loin. Maman revient ? Bientôt. En ce moment, Sarah s'assoit au bas du canapé. Elle pose la feuille sur le tapis. Le crayon jaune fait un bruit sec. Un soleil rond ! Des rayons partent, puis une petite maison. Une porte, deux fenêtres. C'est notre maison. Tu as de la place, Sarah ? Oui, papa. Sarah appuie trop fort, trop vite. Le crayon jaune casse, net. Oh. Il en reste un bout. La mine tombe sur le tapis. Maman va voir le trou ? Elle verra la maison. Sarah veut finir, tout de suite. Je montre, maintenant ! Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois le bout, Sarah ? Oui, papa. L'éclat de gomme tremble, puis tient. Sarah finit le toit avec le bout. Un rayon manque. La maison est là. La porte clique, dans le couloir. Maman pose son sac. Je rentre. Ça sent les crayons. Attends. Sarah attend que maman s'assoie. Ses joues sont chaudes. Elle tend la feuille, sans bousculer. C'est notre maison. Je suis contente. Le soleil est très jaune. On le met où ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>éclat de gomme</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,37 +1321,69 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis inquiétude; intensite=2; destinataire=enfant; sous_texte=elle_veut_montrer_le_soleil_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un rayon traverse la poussière du salon.
-narrateur|Les crayons dorment dans leur boîte en fer.
-narrateur|La boîte est froide, un peu cabossée.
-narrateur|Le tapis sent la laine.
-narrateur|Un coussin a glissé sous la table.
-narrateur|La pendule fait tic, tout bas.
-narrateur|Papa coud un bouton près de la fenêtre.
-narrateur|Maman n'est pas encore rentrée.
-narrateur|Dehors, un vélo passe, très loin.
+          <t>narrateur|La laine du tapis sent le soleil.
+enfant-f|Ça sent la laine, papa.
+papa|Tu la sens, la laine chaude ?
+enfant-f|Oui, papa.
+narrateur|Sarah connaît ce salon, ses recoins.
+narrateur|Cette fin d'après-midi, un coin brille autrement.
+narrateur|La poussière danse près de la table basse.
+enfant-f|Elle danse, papa.
+papa|Tu la vois, près des crayons ?
+enfant-f|Oui.
+narrateur|La boîte en fer est froide, un peu cabossée.
+enfant-f|Elle claque.
+narrateur|Sarah ouvre la boîte près des genoux.
+narrateur|Les crayons roulent, un petit bruit.
 papa|Sarah, tu as choisi une feuille ?
 enfant-f|La grande, blanche.
 enfant-f|C'est pour maman.
-papa|Elle va rentrer bientôt.
+papa|Maman n'est pas rentrée.
+enfant-f|Je lui fais un soleil.
+narrateur|Près de la feuille, un éclat de gomme luit.
+enfant-f|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-f|Oui, un grain blanc.
+narrateur|Papa coud un bouton, près de la fenêtre.
+narrateur|Dehors, un vélo passe, très loin.
+enfant-f|Maman revient ?
+papa|Bientôt.
 narrateur|En ce moment, Sarah s'assoit au bas du canapé.
 narrateur|Elle pose la feuille sur le tapis.
 narrateur|Le crayon jaune fait un bruit sec.
-narrateur|Un soleil rond, puis des rayons.
-narrateur|Une petite maison, une porte, deux fenêtres.
+enfant-f|Un soleil rond !
+narrateur|Des rayons partent, puis une petite maison.
+narrateur|Une porte, deux fenêtres.
+enfant-f|C'est notre maison.
+papa|Tu as de la place, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Sarah appuie trop fort, trop vite.
 narrateur|Le crayon jaune casse, net.
 enfant-f|Oh.
 papa|Il en reste un bout.
-narrateur|Sarah souffle la mine tombée sur le tapis.
-narrateur|Elle finit le toit avec le bout.
-narrateur|Un rayon manque encore, tout petit.
+narrateur|La mine tombe sur le tapis.
 enfant-f|Maman va voir le trou ?
-papa|Elle verra la maison, d'abord.
-narrateur|Sarah pose le bout de crayon.
-narrateur|La porte d'entrée clique.
+papa|Elle verra la maison.
+narrateur|Sarah veut finir, tout de suite.
+enfant-f|Je montre, maintenant !
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois le bout, Sarah ?
+enfant-f|Oui, papa.
+narrateur|L'éclat de gomme tremble, puis tient.
+narrateur|Sarah finit le toit avec le bout.
+enfant-f|Un rayon manque.
+papa|La maison est là.
+narrateur|La porte clique, dans le couloir.
 narrateur|Maman pose son sac.
 maman|Je rentre.
 maman|Ça sent les crayons.
@@ -1361,9 +1393,8 @@
 narrateur|Elle tend la feuille, sans bousculer.
 enfant-f|C'est notre maison.
 enfant-f|Je suis contente.
-maman|Merci, Sarah.
-papa|Le soleil est très jaune.
-maman|On le met où ?</t>
+maman|Le soleil est très jaune.
+papa|On le met où ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1400,12 +1431,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sarah sourit, la feuille encore chaude. Que dit-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Sarah&lt;/emphasis&gt; sourit, la feuille encore chaude. Que dit-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Ninon sourit. Que dit-elle ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Sarah&lt;/emphasis&gt; sourit, la feuille encore chaude. Que dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1468,7 +1499,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1476,10 +1507,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1494,34 +1525,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Sarah</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1530,23 +1565,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=sarah_sourit_la_feuille_chaude_que_dit_elle; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1579,17 +1614,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Maman tient la feuille par les bords. Elle ne plie pas le soleil. Le vrai soleil est à la fenêtre. On va le voir ensemble ? Ils se lèvent. Le sac de maman reste près de la porte. J'apporte la pince à linge ? Oui. Papa prend une pince sur le radiateur. La pince est un peu tiède. Comme le rayon.</t>
+          <t>Maman tient la feuille par les bords. Elle ne plie pas le soleil. Le vrai soleil est à la fenêtre. On va le voir ensemble ? Ils se lèvent. Le sac de maman reste près de la porte. Je le mets, maintenant ! Sarah avance trop vite vers la vitre. Les mots se bousculent dans sa bouche. La pince ! Sarah avance les mains, trop vite. Puis elle s'arrête. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe la feuille, un instant. Elle écoute le salon. Tu restes un peu, Sarah ? Oui, papa. Merci, Sarah. Papa reste à la même hauteur. La feuille est tiède, sous les doigts. Elle est chaude. J'apporte la pince à linge ? Oui. Papa prend une pince sur le radiateur. La pince est un peu tiède. Comme le rayon. Tes mains sont au chaud, Sarah ? Un peu, maman. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. On va près de la vitre ? Oui. On marche sans se presser ? Oui, papa.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Maman tient la feuille par les bords. Elle ne plie pas le soleil. Le vrai soleil est à la fenêtre. On va le voir ensemble ? Ils se lèvent. Le sac de maman reste près de la porte. J'apporte la pince à linge ? Oui. Papa prend une pince sur le radiateur. La pince est un peu tiède. Comme le rayon.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman tient la &lt;emphasis level="moderate"&gt;feuille&lt;/emphasis&gt; par les bords. Elle ne plie pas le soleil. Le vrai soleil est à la fenêtre. On va le voir ensemble ? Ils se lèvent. Le sac de maman reste près de la porte. Je le mets, maintenant ! Sarah avance trop vite vers la vitre. Les mots se bousculent dans sa bouche. La pince ! Sarah avance les mains, trop vite. Puis elle s'arrête. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe la feuille, un instant. Elle écoute le salon. Tu restes un peu, Sarah ? Oui, papa. Merci, Sarah. Papa reste à la même hauteur. La feuille est tiède, sous les doigts. Elle est chaude. J'apporte la pince à linge ? Oui. Papa prend une pince sur le radiateur. La pince est un peu tiède. Comme le rayon. Tes mains sont au chaud, Sarah ? Un peu, maman. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. On va près de la vitre ? Oui. On marche sans se presser ? Oui, papa.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ninon a nommé sa joie. Elle a partagé avec papa et maman. Être &lt;emphasis&gt;content&lt;/emphasis&gt;, c'est bien. [pause]</t>
+          <t>Maman tient la &lt;emphasis&gt;feuille&lt;/emphasis&gt; par les bords. Elle ne plie pas le soleil. Le vrai soleil est à la fenêtre. On va le voir ensemble ? Ils se lèvent. Le sac de maman reste près de la porte. Je le mets, maintenant ! Sarah avance trop vite vers la vitre. Les mots se bousculent dans sa bouche. La pince ! Sarah avance les mains, trop vite. Puis elle s'arrête. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe la feuille, un instant. Elle écoute le salon. Tu restes un peu, Sarah ? Oui, papa. Merci, Sarah. Papa reste à la même hauteur. La feuille est tiède, sous les doigts. Elle est chaude. J'apporte la pince à linge ? Oui. Papa prend une pince sur le radiateur. La pince est un peu tiède. Comme le rayon. Tes mains sont au chaud, Sarah ? Un peu, maman. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. On va près de la vitre ? Oui. On marche sans se presser ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1636,7 +1671,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1644,10 +1679,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1670,30 +1705,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>feuille</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1702,10 +1737,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1718,7 +1753,7 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_attend_elle_montre_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
@@ -1729,11 +1764,36 @@
 maman|On va le voir ensemble ?
 narrateur|Ils se lèvent.
 narrateur|Le sac de maman reste près de la porte.
+enfant-f|Je le mets, maintenant !
+narrateur|Sarah avance trop vite vers la vitre.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|La pince !
+narrateur|Sarah avance les mains, trop vite.
+narrateur|Puis elle s'arrête.
+narrateur|Sarah refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe la feuille, un instant.
+narrateur|Elle écoute le salon.
+papa|Tu restes un peu, Sarah ?
+enfant-f|Oui, papa.
+papa|Merci, Sarah.
+narrateur|Papa reste à la même hauteur.
+maman|La feuille est tiède, sous les doigts.
+enfant-f|Elle est chaude.
 papa|J'apporte la pince à linge ?
 enfant-f|Oui.
 narrateur|Papa prend une pince sur le radiateur.
 narrateur|La pince est un peu tiède.
-enfant-f|Comme le rayon.</t>
+enfant-f|Comme le rayon.
+maman|Tes mains sont au chaud, Sarah ?
+enfant-f|Un peu, maman.
+narrateur|Le ventre de Sarah se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On va près de la vitre ?
+enfant-f|Oui.
+papa|On marche sans se presser ?
+enfant-f|Oui, papa.</t>
         </is>
       </c>
     </row>
@@ -1760,17 +1820,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils collent le dessin contre la vitre. La pince tient le coin. Dehors, le vrai soleil est plus pâle. Le mien est plus rond. Le tien attendait, sur le tapis. Le crayon cassé reste dans la boîte. Sarah range les autres crayons, un par un. Le jaune cassé rentre le dernier. La boîte fait un petit clac. On laisse le dessin pour la nuit ? Oui. Il garde la fenêtre.</t>
+          <t>Ils collent le dessin contre la vitre. La pince tient le coin. Il garde la fenêtre. Sarah pousse trop vite, tout de suite. La feuille se plie, net. Elle plie ! Un coin se recroqueville contre la vitre. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la feuille, un instant. Elle écoute le salon, près de la vitre. Sur le papier, un éclat de gomme luit. Là, sur le papier. Sarah lisse le pli, sans se presser. On tient le coin ? Oui, papa. La pince reprend le bord. La feuille se déplie. Poumf. Le soleil est à sa place, Sarah ? Oui, maman. Dehors, le vrai soleil est plus pâle. Le mien est plus rond. Le tien attendait, sur le tapis. Le crayon cassé reste dans la boîte. Sarah range les autres crayons, un par un. Le jaune cassé rentre le dernier. La boîte fait un petit clac. On laisse le dessin pour la nuit ? Oui. Il garde la fenêtre. Tu vois le point, Sarah ? Oui, papa.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ils collent le dessin contre la vitre. La pince tient le coin. Dehors, le vrai soleil est plus pâle. Le mien est plus rond. Le tien attendait, sur le tapis. Le crayon cassé reste dans la boîte. Sarah range les autres crayons, un par un. Le jaune cassé rentre le dernier. La boîte fait un petit clac. On laisse le dessin pour la nuit ? Oui. Il garde la fenêtre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils collent le dessin contre la vitre. La pince tient le coin. Il garde la fenêtre. Sarah pousse trop vite, tout de suite. La feuille se plie, net. Elle plie ! Un coin se recroqueville contre la vitre. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la feuille, un instant. Elle écoute le salon, près de la vitre. Sur le papier, un &lt;emphasis level="moderate"&gt;éclat de gomme&lt;/emphasis&gt; luit. Là, sur le papier. Sarah lisse le pli, sans se presser. On tient le coin ? Oui, papa. La pince reprend le bord. La feuille se déplie. Poumf. Le soleil est à sa place, Sarah ? Oui, maman. Dehors, le vrai soleil est plus pâle. Le mien est plus rond. Le tien attendait, sur le tapis. Le crayon cassé reste dans la boîte. Sarah range les autres crayons, un par un. Le jaune cassé rentre le dernier. La boîte fait un petit clac. On laisse le dessin pour la nuit ? Oui. Il garde la fenêtre. Tu vois le point, Sarah ? Oui, papa.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Ninon range ses crayons. Le salon est calme. Papa lui prend la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Ils collent le dessin contre la vitre. La pince tient le coin. Il garde la fenêtre. Sarah pousse trop vite, tout de suite. La feuille se plie, net. Elle plie ! Un coin se recroqueville contre la vitre. Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la feuille, un instant. Elle écoute le salon, près de la vitre. Sur le papier, un &lt;emphasis&gt;éclat de gomme&lt;/emphasis&gt; luit. Là, sur le papier. Sarah lisse le pli, sans se presser. On tient le coin ? Oui, papa. La pince reprend le bord. La feuille se déplie. Poumf. Le soleil est à sa place, Sarah ? Oui, maman. Dehors, le vrai soleil est plus pâle. Le mien est plus rond. Le tien attendait, sur le tapis. Le crayon cassé reste dans la boîte. Sarah range les autres crayons, un par un. Le jaune cassé rentre le dernier. La boîte fait un petit clac. On laisse le dessin pour la nuit ? Oui. Il garde la fenêtre. Tu vois le point, Sarah ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1817,7 +1877,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1825,10 +1885,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1851,30 +1911,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de gomme</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1883,10 +1943,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1897,12 +1957,38 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=la_feuille_se_plie_elle_refuse_de_foncer; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
           <t>narrateur|Ils collent le dessin contre la vitre.
 narrateur|La pince tient le coin.
-narrateur|Dehors, le vrai soleil est plus pâle.
+enfant-f|Il garde la fenêtre.
+narrateur|Sarah pousse trop vite, tout de suite.
+narrateur|La feuille se plie, net.
+enfant-f|Elle plie !
+narrateur|Un coin se recroqueville contre la vitre.
+narrateur|Sarah avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Sarah refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe la feuille, un instant.
+narrateur|Elle écoute le salon, près de la vitre.
+narrateur|Sur le papier, un éclat de gomme luit.
+enfant-f|Là, sur le papier.
+narrateur|Sarah lisse le pli, sans se presser.
+papa|On tient le coin ?
+enfant-f|Oui, papa.
+narrateur|La pince reprend le bord.
+narrateur|La feuille se déplie.
+enfant-f|Poumf.
+maman|Le soleil est à sa place, Sarah ?
+enfant-f|Oui, maman.
+papa|Dehors, le vrai soleil est plus pâle.
 enfant-f|Le mien est plus rond.
 maman|Le tien attendait, sur le tapis.
 papa|Le crayon cassé reste dans la boîte.
@@ -1911,7 +1997,9 @@
 narrateur|La boîte fait un petit clac.
 papa|On laisse le dessin pour la nuit ?
 enfant-f|Oui.
-enfant-f|Il garde la fenêtre.</t>
+enfant-f|Il garde la fenêtre.
+papa|Tu vois le point, Sarah ?
+enfant-f|Oui, papa.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1943,17 +2031,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le rayon a bougé sur le tapis. Sur la vitre, la maison reste. Maman l'a vue. Je la verrai encore demain. Le sac de maman sent encore le dehors. Ils restent au salon, tout près.</t>
+          <t>Ils restent près de la vitre. Maman essuie un peu de poussière. Maman a vu la maison, papa. Tu l'as vue, toi ? Oui, près du soleil. On est bien, ici. Sarah tapote le papier du doigt. Il a une trace de crayon. Tu la vois, la trace ? Oui, maman. Le dessin est resté, Sarah. Oui, avec le soleil. Ça sent les crayons, un peu tièdes. Et la laine, maman. Oui, dans l'air. Le salon est calme, Sarah ? Oui, papa. Le dessin reste contre la vitre. Un éclat de gomme tient sur le papier.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le rayon a bougé sur le tapis. Sur la vitre, la maison reste. Maman l'a vue. Je la verrai encore demain. Le sac de maman sent encore le dehors. Ils restent au salon, tout près.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la vitre. Maman essuie un peu de poussière. Maman a vu la maison, papa. Tu l'as vue, toi ? Oui, près du soleil. On est bien, ici. Sarah tapote le papier du doigt. Il a une trace de crayon. Tu la vois, la trace ? Oui, maman. Le dessin est resté, Sarah. Oui, avec le soleil. Ça sent les crayons, un peu tièdes. Et la laine, maman. Oui, dans l'air. Le salon est calme, Sarah ? Oui, papa. Le dessin reste contre la vitre. Un &lt;emphasis level="moderate"&gt;éclat de gomme&lt;/emphasis&gt; tient sur le papier.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la vitre. Maman essuie un peu de poussière. Maman a vu la maison, papa. Tu l'as vue, toi ? Oui, près du soleil. On est bien, ici. Sarah tapote le papier du doigt. Il a une trace de crayon. Tu la vois, la trace ? Oui, maman. Le dessin est resté, Sarah. Oui, avec le soleil. Ça sent les crayons, un peu tièdes. Et la laine, maman. Oui, dans l'air. Le salon est calme, Sarah ? Oui, papa. Le dessin reste contre la vitre. Un &lt;emphasis&gt;éclat de gomme&lt;/emphasis&gt; tient sur le papier.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2000,18 +2088,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2020,12 +2108,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2034,17 +2122,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de gomme</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2053,11 +2145,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2066,29 +2158,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_papier; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le rayon a bougé sur le tapis.
-narrateur|Sur la vitre, la maison reste.
-enfant-f|Maman l'a vue.
-maman|Je la verrai encore demain.
-narrateur|Le sac de maman sent encore le dehors.
-narrateur|Ils restent au salon, tout près.</t>
+          <t>narrateur|Ils restent près de la vitre.
+narrateur|Maman essuie un peu de poussière.
+enfant-f|Maman a vu la maison, papa.
+papa|Tu l'as vue, toi ?
+enfant-f|Oui, près du soleil.
+maman|On est bien, ici.
+narrateur|Sarah tapote le papier du doigt.
+enfant-f|Il a une trace de crayon.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|Le dessin est resté, Sarah.
+enfant-f|Oui, avec le soleil.
+narrateur|Ça sent les crayons, un peu tièdes.
+enfant-f|Et la laine, maman.
+maman|Oui, dans l'air.
+papa|Le salon est calme, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Le dessin reste contre la vitre.
+narrateur|Un éclat de gomme tient sur le papier.</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2180,6 +2289,13 @@
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>